<commit_message>
Bank reconciliation: reconciliation start date, printable statement layout
- Book entries dated before a bank account's reconciliation start (bank account
  master reconcileFrom, else the first statement's start date) are covered by the
  first statement's opening balance and left out of the book side, so a go-live with
  earlier GL history reconciles; settable on the bank account setup until a
  reconciliation is approved.
- The PDF statement prints each side as an aligned figures table and keeps the
  Latin-1 text readable; workspace panes fit the status under the amount.
</commit_message>
<xml_diff>
--- a/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
+++ b/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
@@ -1332,7 +1332,7 @@
     <t xml:space="preserve">/api/bank-reconciliation/bank-accounts/:code</t>
   </si>
   <si>
-    <t xml:space="preserve">Link a bank account to its GL cash account and default statement format (stored on the bank account master record)</t>
+    <t xml:space="preserve">Link a bank account to its GL cash account, default statement format and reconciliation start date (book entries before it are covered by the first statement's opening balance; default: the first statement's start)</t>
   </si>
   <si>
     <t xml:space="preserve">Accounts &gt; Bank Reconciliation &gt; Bank account setup</t>
@@ -1340,7 +1340,8 @@
   <si>
     <t xml:space="preserve">{
   "glAccountCode": "1102001",
-  "statementFormat": "BDO-SAMPLE"
+  "statementFormat": "BDO-SAMPLE",
+  "reconcileFrom": "2026-08-01"
 }</t>
   </si>
   <si>
@@ -1348,7 +1349,8 @@
   "success": true,
   "data": {
     "code": "ACC-BDO-001",
-    "glAccountCode": "1102001"
+    "glAccountCode": "1102001",
+    "reconcileFrom": "2026-08-01"
   }
 }</t>
   </si>

</xml_diff>

<commit_message>
Add the deployment guide content, environment templates, CI and pipeline changes
The previous commit only moved the deployment documents. This adds their updated content, the environment
templates with placeholders, the repository CI workflow, the front-end deploy workflow (Node 22, tests first, API
address required) and the API documents with the corrected route addresses.
</commit_message>
<xml_diff>
--- a/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
+++ b/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9866" uniqueCount="2797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9866" uniqueCount="2798">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -56,7 +56,7 @@
     <t xml:space="preserve">GET</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/posting-rules/account-determination</t>
+    <t xml:space="preserve">/api/account-determination</t>
   </si>
   <si>
     <t xml:space="preserve">Account roles the posting rules use (by section), payable account per payee type, cash account per payment mode, write-off reasons</t>
@@ -110,7 +110,7 @@
     <t xml:space="preserve">PUT</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/posting-rules/account-determination/maps/:name</t>
+    <t xml:space="preserve">/api/account-determination/maps/:name</t>
   </si>
   <si>
     <t xml:space="preserve">Replace the payable account per payee type (payable-by-payee) or the cash account per payment mode (cash-by-payment-mode)</t>
@@ -136,7 +136,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/posting-rules/account-determination/roles/:role</t>
+    <t xml:space="preserve">/api/account-determination/roles/:role</t>
   </si>
   <si>
     <t xml:space="preserve">Set the GL account of an account role (accounting.account.&lt;role&gt;) used by the posting rules</t>
@@ -157,7 +157,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/posting-rules/account-determination/write-off-reasons</t>
+    <t xml:space="preserve">/api/account-determination/write-off-reasons</t>
   </si>
   <si>
     <t xml:space="preserve">Write-off reasons with their GL account (all statuses)</t>
@@ -204,7 +204,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/posting-rules/account-determination/write-off-reasons/:code</t>
+    <t xml:space="preserve">/api/account-determination/write-off-reasons/:code</t>
   </si>
   <si>
     <t xml:space="preserve">Update a write-off reason (name, GL account, limit, status)</t>
@@ -2347,7 +2347,7 @@
     <t xml:space="preserve">Billing statements</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/receipts/billing-statement/endorsement/:id/generate</t>
+    <t xml:space="preserve">/api/billing-statement/endorsement/:id/generate</t>
   </si>
   <si>
     <t xml:space="preserve">Endorsement billing statement (PDF); id = endorsement or policy id</t>
@@ -2359,7 +2359,7 @@
     <t xml:space="preserve">read:policies, read:receipts</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/receipts/billing-statement/endorsement/:id/preview</t>
+    <t xml:space="preserve">/api/billing-statement/endorsement/:id/preview</t>
   </si>
   <si>
     <t xml:space="preserve">Endorsement billing preview (JSON); id = endorsement or policy id</t>
@@ -2382,7 +2382,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/receipts/billing-statement/policy/:policyId/generate</t>
+    <t xml:space="preserve">/api/billing-statement/policy/:policyId/generate</t>
   </si>
   <si>
     <t xml:space="preserve">Policy billing statement (PDF)</t>
@@ -2391,7 +2391,7 @@
     <t xml:space="preserve">Agent &gt; Policy detail &gt; Generate invoice (policy)</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/receipts/billing-statement/renewal/:policyId/generate</t>
+    <t xml:space="preserve">/api/billing-statement/renewal/:policyId/generate</t>
   </si>
   <si>
     <t xml:space="preserve">Renewal billing statement (PDF)</t>
@@ -2403,7 +2403,7 @@
     <t xml:space="preserve">Broker Slips</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips</t>
+    <t xml:space="preserve">/api/broker-slips</t>
   </si>
   <si>
     <t xml:space="preserve">List broker slips (status (comma-separated), lob, leadRefId, clientId, insurerId, search; paging) with offer counts and status counts</t>
@@ -2519,7 +2519,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id</t>
+    <t xml:space="preserve">/api/broker-slips/:id</t>
   </si>
   <si>
     <t xml:space="preserve">Broker slip with insurer offers, comparison (ranked by gross premium, capacity), journey and links</t>
@@ -2610,7 +2610,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/cancel</t>
+    <t xml:space="preserve">/api/broker-slips/:id/cancel</t>
   </si>
   <si>
     <t xml:space="preserve">Cancel the broker slip</t>
@@ -2651,7 +2651,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/close</t>
+    <t xml:space="preserve">/api/broker-slips/:id/close</t>
   </si>
   <si>
     <t xml:space="preserve">Close the broker slip without a quotation (e.g. not taken up)</t>
@@ -2687,7 +2687,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/comparison</t>
+    <t xml:space="preserve">/api/broker-slips/:id/comparison</t>
   </si>
   <si>
     <t xml:space="preserve">Comparison of the insurer offers (ranked by gross premium, difference from the best, market capacity)</t>
@@ -2722,7 +2722,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/documents/broker-slip</t>
+    <t xml:space="preserve">/api/broker-slips/:id/documents/broker-slip</t>
   </si>
   <si>
     <t xml:space="preserve">Broker Slip PDF (request for quotation); insurerId= addresses it to one insurer of the market</t>
@@ -2737,7 +2737,7 @@
     <t xml:space="preserve">application/pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/insurers</t>
+    <t xml:space="preserve">/api/broker-slips/:id/insurers</t>
   </si>
   <si>
     <t xml:space="preserve">Approach one more insurer (on a submitted slip the request is queued at once)</t>
@@ -2781,7 +2781,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/offers/:offerId</t>
+    <t xml:space="preserve">/api/broker-slips/:id/offers/:offerId</t>
   </si>
   <si>
     <t xml:space="preserve">Record an insurer's response: offer (premium, rate, taxes, deductibles, terms, validity, line %, reference, attachment) or decline</t>
@@ -2818,7 +2818,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/prepare-placement</t>
+    <t xml:space="preserve">/api/broker-slips/:id/prepare-placement</t>
   </si>
   <si>
     <t xml:space="preserve">Prepare the Placement Slip straight from the selected offer(s) (journeys where the Quotation Slip is optional or skipped)</t>
@@ -2846,7 +2846,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/prepare-quotation</t>
+    <t xml:space="preserve">/api/broker-slips/:id/prepare-quotation</t>
   </si>
   <si>
     <t xml:space="preserve">Prepare the Quotation Slip from the selected offer(s): several offers make it co-insurance with their lines as shares (must total 100%)</t>
@@ -2873,7 +2873,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/placements/broker-slips/:id/submit</t>
+    <t xml:space="preserve">/api/broker-slips/:id/submit</t>
   </si>
   <si>
     <t xml:space="preserve">Submit the broker slip to the market: queues the request for quotation to each insurer (outbox) and sets the response due date</t>
@@ -3719,7 +3719,21 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/clients/customers/codes</t>
+    <t xml:space="preserve">/api/clients/from-lead/:leadId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convert a lead into a client (returns the existing client when already converted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations &gt; Quotation &gt; Convert to policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "contactNumber": "09171234567"
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/api/customers/codes</t>
   </si>
   <si>
     <t xml:space="preserve">Customer codes for dropdowns</t>
@@ -3737,20 +3751,6 @@
       "name": "Juan Dela Cruz"
     }
   ]
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/clients/from-lead/:leadId</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Convert a lead into a client (returns the existing client when already converted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations &gt; Quotation &gt; Convert to policy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "contactNumber": "09171234567"
 }</t>
   </si>
   <si>
@@ -5516,7 +5516,7 @@
     <t xml:space="preserve">E-mail</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/email/generate</t>
+    <t xml:space="preserve">/api/email/generate</t>
   </si>
   <si>
     <t xml:space="preserve">Generate e-mail content (subject, preview, html, text) for a quote from the configured template</t>
@@ -5551,7 +5551,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/email/send</t>
+    <t xml:space="preserve">/api/email/send</t>
   </si>
   <si>
     <t xml:space="preserve">Send an e-mail composed in the Share dialog</t>
@@ -5573,7 +5573,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/email/share-quote</t>
+    <t xml:space="preserve">/api/email/share-quote</t>
   </si>
   <si>
     <t xml:space="preserve">E-mail a quotation to a recipient with the standard template</t>
@@ -5597,7 +5597,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/email/share-quote-to-insurers</t>
+    <t xml:space="preserve">/api/email/share-quote-to-insurers</t>
   </si>
   <si>
     <t xml:space="preserve">Send the quotation to selected insurers (contact e-mail from the insurance company master)</t>
@@ -6020,7 +6020,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/s3/upload/file/*</t>
+    <t xml:space="preserve">/api/upload/file/*</t>
   </si>
   <si>
     <t xml:space="preserve">Download a stored file (older link form of /s3/object)</t>
@@ -7020,16 +7020,54 @@
     <t xml:space="preserve">Leads</t>
   </si>
   <si>
+    <t xml:space="preserve">/api/lead/get-all-lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy: list leads (same as GET /leads)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations &gt; Leads/Prospects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">read:leads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "success": true,
+  "data": [
+    {
+      "leadId": "ld_1",
+      "generatedLeadId": "LD-2026-00001",
+      "firstName": "Juan",
+      "lastName": "Dela Cruz",
+      "leadCategory": "Retail",
+      "lob": "MOTOR",
+      "emailId": "juan@example.com",
+      "contactNumber": "09171234567",
+      "city": "Makati",
+      "province": "Metro Manila",
+      "country": "Philippines",
+      "status": "New",
+      "quotationsCount": 0
+    }
+  ],
+  "total": 1
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/api/lead/search-lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy: search leads by name (same as GET /leads/search)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Query: ?name=juan</t>
+  </si>
+  <si>
     <t xml:space="preserve">/api/leads</t>
   </si>
   <si>
     <t xml:space="preserve">List leads (filters leadCategory, country, province, city, lob, status; search query; paging)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations &gt; Leads/Prospects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">read:leads</t>
   </si>
   <si>
     <t xml:space="preserve">Query: ?page=1&amp;pageSize=10&amp;leadCategory=Retail&amp;lob=FIRE&amp;query=juan</t>
@@ -7181,44 +7219,6 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/leads/lead/get-all-lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy: list leads (same as GET /leads)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "success": true,
-  "data": [
-    {
-      "leadId": "ld_1",
-      "generatedLeadId": "LD-2026-00001",
-      "firstName": "Juan",
-      "lastName": "Dela Cruz",
-      "leadCategory": "Retail",
-      "lob": "MOTOR",
-      "emailId": "juan@example.com",
-      "contactNumber": "09171234567",
-      "city": "Makati",
-      "province": "Metro Manila",
-      "country": "Philippines",
-      "status": "New",
-      "quotationsCount": 0
-    }
-  ],
-  "total": 1
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/leads/lead/search-lead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legacy: search leads by name (same as GET /leads/search)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Query: ?name=juan</t>
-  </si>
-  <si>
     <t xml:space="preserve">/api/leads/report</t>
   </si>
   <si>
@@ -7537,7 +7537,7 @@
     <t xml:space="preserve">Notifications</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications</t>
+    <t xml:space="preserve">/api/notifications</t>
   </si>
   <si>
     <t xml:space="preserve">Notifications for the signed-in user (paged; filter type / isRead)</t>
@@ -7589,19 +7589,19 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/:id</t>
+    <t xml:space="preserve">/api/notifications/:id</t>
   </si>
   <si>
     <t xml:space="preserve">Delete one notification</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/:id/read</t>
+    <t xml:space="preserve">/api/notifications/:id/read</t>
   </si>
   <si>
     <t xml:space="preserve">Mark one notification as read</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/read</t>
+    <t xml:space="preserve">/api/notifications/read</t>
   </si>
   <si>
     <t xml:space="preserve">Mark several notifications as read</t>
@@ -7615,7 +7615,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/read-all</t>
+    <t xml:space="preserve">/api/notifications/read-all</t>
   </si>
   <si>
     <t xml:space="preserve">Mark all notifications as read</t>
@@ -7629,7 +7629,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/stats</t>
+    <t xml:space="preserve">/api/notifications/stats</t>
   </si>
   <si>
     <t xml:space="preserve">Notification totals by type</t>
@@ -7644,7 +7644,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/accounting/notifications/unread-count</t>
+    <t xml:space="preserve">/api/notifications/unread-count</t>
   </si>
   <si>
     <t xml:space="preserve">Unread notification count</t>
@@ -7662,7 +7662,7 @@
     <t xml:space="preserve">Open Items</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/open-items</t>
+    <t xml:space="preserve">/api/open-items</t>
   </si>
   <si>
     <t xml:space="preserve">Open items: pending payments, renewal requests, pending quotes, expiring policies (filter type, search)</t>
@@ -7704,7 +7704,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/open-items/events</t>
+    <t xml:space="preserve">/api/open-items/events</t>
   </si>
   <si>
     <t xml:space="preserve">Upcoming events of the signed-in user</t>
@@ -7753,7 +7753,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/open-items/events/:id</t>
+    <t xml:space="preserve">/api/open-items/events/:id</t>
   </si>
   <si>
     <t xml:space="preserve">Remove one of the signed-in user's events</t>
@@ -8676,7 +8676,7 @@
     <t xml:space="preserve">Petty Cash</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/disbursements</t>
+    <t xml:space="preserve">/api/petty-cash/disbursements</t>
   </si>
   <si>
     <t xml:space="preserve">Petty cash disbursements (search, fundId / pettyCashCode, status; paging)</t>
@@ -8741,7 +8741,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/disbursements/:id</t>
+    <t xml:space="preserve">/api/petty-cash/disbursements/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One petty cash disbursement (id or number)</t>
@@ -8750,7 +8750,7 @@
     <t xml:space="preserve">Accounts &gt; Petty Cash &gt; Disbursement &gt; View</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/disbursements/:id/reverse</t>
+    <t xml:space="preserve">/api/petty-cash/disbursements/:id/reverse</t>
   </si>
   <si>
     <t xml:space="preserve">Reverse a petty cash disbursement entered in error (mirror journal, fund cash restored)</t>
@@ -8773,7 +8773,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/funds</t>
+    <t xml:space="preserve">/api/petty-cash/funds</t>
   </si>
   <si>
     <t xml:space="preserve">Petty cash funds (search, fundId / pettyCashCode, status; paging)</t>
@@ -8835,7 +8835,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/funds/:id</t>
+    <t xml:space="preserve">/api/petty-cash/funds/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One petty cash fund (id or number)</t>
@@ -8855,7 +8855,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/receipts</t>
+    <t xml:space="preserve">/api/petty-cash/receipts</t>
   </si>
   <si>
     <t xml:space="preserve">Petty cash receipts (search, fundId / pettyCashCode, status; paging)</t>
@@ -8908,7 +8908,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/receipts/:id</t>
+    <t xml:space="preserve">/api/petty-cash/receipts/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One petty cash receipt (id or number)</t>
@@ -8917,13 +8917,13 @@
     <t xml:space="preserve">Accounts &gt; Petty Cash &gt; Receipts &gt; View</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/receipts/:id/reverse</t>
+    <t xml:space="preserve">/api/petty-cash/receipts/:id/reverse</t>
   </si>
   <si>
     <t xml:space="preserve">Reverse a petty cash receipt entered in error (mirror journal, fund cash restored)</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/replenishments</t>
+    <t xml:space="preserve">/api/petty-cash/replenishments</t>
   </si>
   <si>
     <t xml:space="preserve">Petty cash replenishments (search, fundId / pettyCashCode, status; paging)</t>
@@ -8970,7 +8970,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/replenishments/:id</t>
+    <t xml:space="preserve">/api/petty-cash/replenishments/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One petty cash replenishment (id or number)</t>
@@ -8979,13 +8979,13 @@
     <t xml:space="preserve">Accounts &gt; Petty Cash &gt; Replenish &gt; View</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/replenishments/:id/reverse</t>
+    <t xml:space="preserve">/api/petty-cash/replenishments/:id/reverse</t>
   </si>
   <si>
     <t xml:space="preserve">Reverse a petty cash replenishment entered in error (mirror journal, fund cash restored)</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/requests</t>
+    <t xml:space="preserve">/api/petty-cash/requests</t>
   </si>
   <si>
     <t xml:space="preserve">Petty cash requests (search, fundId / pettyCashCode, status; paging)</t>
@@ -9059,7 +9059,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/requests/:id</t>
+    <t xml:space="preserve">/api/petty-cash/requests/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One petty cash request (id or number)</t>
@@ -9089,7 +9089,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/requests/:id/approve</t>
+    <t xml:space="preserve">/api/petty-cash/requests/:id/approve</t>
   </si>
   <si>
     <t xml:space="preserve">Approve a submitted request (approver must differ from requester)</t>
@@ -9114,7 +9114,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/requests/:id/reject</t>
+    <t xml:space="preserve">/api/petty-cash/requests/:id/reject</t>
   </si>
   <si>
     <t xml:space="preserve">Reject a submitted request (approver must differ from requester)</t>
@@ -9144,7 +9144,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/payments/petty-cash/requests/:id/submit</t>
+    <t xml:space="preserve">/api/petty-cash/requests/:id/submit</t>
   </si>
   <si>
     <t xml:space="preserve">Submit a request for approval</t>
@@ -12249,7 +12249,7 @@
     <t xml:space="preserve">Quotation masters</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/biCoverage/get-bi-coverage</t>
+    <t xml:space="preserve">/api/biCoverage/get-bi-coverage</t>
   </si>
   <si>
     <t xml:space="preserve">BI coverage options (amount and flat premium) for a policy type</t>
@@ -12277,7 +12277,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/account-codes</t>
+    <t xml:space="preserve">/api/master/account-codes</t>
   </si>
   <si>
     <t xml:space="preserve">Account codes for a quote: active referrers (agents, sub-agents, external) as dropdown options</t>
@@ -12297,7 +12297,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/banks/get-all-banks</t>
+    <t xml:space="preserve">/api/master/banks/get-all-banks</t>
   </si>
   <si>
     <t xml:space="preserve">Banks / mortgagees</t>
@@ -12318,7 +12318,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/insurancecompany/get-insurance-companies</t>
+    <t xml:space="preserve">/api/master/insurancecompany/get-insurance-companies</t>
   </si>
   <si>
     <t xml:space="preserve">Insurance companies</t>
@@ -12337,7 +12337,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/policyType/policy-type</t>
+    <t xml:space="preserve">/api/master/policyType/policy-type</t>
   </si>
   <si>
     <t xml:space="preserve">Policy types of a product (productId = id or code)</t>
@@ -12359,7 +12359,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/signatory/get-all-signatory</t>
+    <t xml:space="preserve">/api/master/signatory/get-all-signatory</t>
   </si>
   <si>
     <t xml:space="preserve">Authorised signatories</t>
@@ -12380,7 +12380,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/vehicle/get-brands</t>
+    <t xml:space="preserve">/api/master/vehicle/get-brands</t>
   </si>
   <si>
     <t xml:space="preserve">Vehicle brands</t>
@@ -12398,7 +12398,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/vehicle/get-models</t>
+    <t xml:space="preserve">/api/master/vehicle/get-models</t>
   </si>
   <si>
     <t xml:space="preserve">Models of a brand (brand id or name)</t>
@@ -12420,7 +12420,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/vehicle/get-seating-capacity</t>
+    <t xml:space="preserve">/api/master/vehicle/get-seating-capacity</t>
   </si>
   <si>
     <t xml:space="preserve">Seating capacities (optionally of one variant)</t>
@@ -12441,7 +12441,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/vehicle/get-variants</t>
+    <t xml:space="preserve">/api/master/vehicle/get-variants</t>
   </si>
   <si>
     <t xml:space="preserve">Variants of a model (model id or name)</t>
@@ -12464,7 +12464,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/master/vehicle/get-vehicle-types</t>
+    <t xml:space="preserve">/api/master/vehicle/get-vehicle-types</t>
   </si>
   <si>
     <t xml:space="preserve">Vehicle body types (from the variants master)</t>
@@ -12481,19 +12481,19 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/paCoverage/get-pa-coverages</t>
+    <t xml:space="preserve">/api/paCoverage/get-pa-coverages</t>
   </si>
   <si>
     <t xml:space="preserve">PA coverage options (amount and flat premium) for a policy type</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/pdCoverage/get-pd-coverages</t>
+    <t xml:space="preserve">/api/pdCoverage/get-pd-coverages</t>
   </si>
   <si>
     <t xml:space="preserve">PD coverage options (amount and flat premium) for a policy type</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/quotations/quote/calculate-premium-quote</t>
+    <t xml:space="preserve">/api/quote/calculate-premium-quote</t>
   </si>
   <si>
     <t xml:space="preserve">Legacy premium calculation (same as POST /quotations/calculate-premium)</t>
@@ -16709,7 +16709,7 @@
     <t xml:space="preserve">Renewals workspace</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id</t>
+    <t xml:space="preserve">/api/renewals/:id</t>
   </si>
   <si>
     <t xml:space="preserve">Operations &gt; Renewals &gt; Renewal Queue &gt; View</t>
@@ -16748,7 +16748,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/activities</t>
+    <t xml:space="preserve">/api/renewals/:id/activities</t>
   </si>
   <si>
     <t xml:space="preserve">Add a negotiation update / contact to the renewal timeline</t>
@@ -16778,7 +16778,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/approve</t>
+    <t xml:space="preserve">/api/renewals/:id/approve</t>
   </si>
   <si>
     <t xml:space="preserve">Checker decision on renewal terms (decision approve | reject); approver must differ from the submitter</t>
@@ -16823,7 +16823,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/complete</t>
+    <t xml:space="preserve">/api/renewals/:id/complete</t>
   </si>
   <si>
     <t xml:space="preserve">Complete the renewal: create the new policy term, mark the old policy renewed, raise the premium receivable</t>
@@ -16877,7 +16877,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/lapse</t>
+    <t xml:space="preserve">/api/renewals/:id/lapse</t>
   </si>
   <si>
     <t xml:space="preserve">Lapse a renewal (reason required)</t>
@@ -16921,7 +16921,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/notices</t>
+    <t xml:space="preserve">/api/renewals/:id/notices</t>
   </si>
   <si>
     <t xml:space="preserve">Send the next renewal notice (first, second, final in order); stage may be given explicitly</t>
@@ -16963,7 +16963,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/quote</t>
+    <t xml:space="preserve">/api/renewals/:id/quote</t>
   </si>
   <si>
     <t xml:space="preserve">Generate a renewal quote re-rated at current rates (claims loading, loyalty discount, current taxes) with premium variance</t>
@@ -16997,7 +16997,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/reinstate</t>
+    <t xml:space="preserve">/api/renewals/:id/reinstate</t>
   </si>
   <si>
     <t xml:space="preserve">Reinstate a lapsed renewal within the reinstatement window</t>
@@ -17038,7 +17038,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/reminders</t>
+    <t xml:space="preserve">/api/renewals/:id/reminders</t>
   </si>
   <si>
     <t xml:space="preserve">Send / log a renewal reminder (Email | SMS | Phone | Letter)</t>
@@ -17083,7 +17083,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/submit</t>
+    <t xml:space="preserve">/api/renewals/:id/submit</t>
   </si>
   <si>
     <t xml:space="preserve">Submit the quoted renewal terms for checker approval</t>
@@ -17124,7 +17124,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/:id/win-back</t>
+    <t xml:space="preserve">/api/renewals/:id/win-back</t>
   </si>
   <si>
     <t xml:space="preserve">Record a win-back offer on a lapsed renewal (optionally linked to a campaign)</t>
@@ -17147,7 +17147,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/approvals</t>
+    <t xml:space="preserve">/api/renewals/approvals</t>
   </si>
   <si>
     <t xml:space="preserve">Renewal terms awaiting checker approval</t>
@@ -17175,7 +17175,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/at-risk</t>
+    <t xml:space="preserve">/api/renewals/at-risk</t>
   </si>
   <si>
     <t xml:space="preserve">At-risk renewals: risk score, factors, recommended actions</t>
@@ -17211,7 +17211,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/campaigns</t>
+    <t xml:space="preserve">/api/renewals/campaigns</t>
   </si>
   <si>
     <t xml:space="preserve">Win-back campaigns with statistics</t>
@@ -17264,7 +17264,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/campaigns/:id</t>
+    <t xml:space="preserve">/api/renewals/campaigns/:id</t>
   </si>
   <si>
     <t xml:space="preserve">One win-back campaign</t>
@@ -17278,7 +17278,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/lapsed</t>
+    <t xml:space="preserve">/api/renewals/lapsed</t>
   </si>
   <si>
     <t xml:space="preserve">Lapsed renewals with win-back attempts and reinstatement eligibility</t>
@@ -17301,7 +17301,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/negotiations</t>
+    <t xml:space="preserve">/api/renewals/negotiations</t>
   </si>
   <si>
     <t xml:space="preserve">Renewals under negotiation with their contact timeline</t>
@@ -17332,7 +17332,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/performance</t>
+    <t xml:space="preserve">/api/renewals/performance</t>
   </si>
   <si>
     <t xml:space="preserve">Retention KPIs: renewal rate, premium retention, cycle time, by product, by agent, monthly trend</t>
@@ -17379,7 +17379,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/pipeline/refresh</t>
+    <t xml:space="preserve">/api/renewals/pipeline/refresh</t>
   </si>
   <si>
     <t xml:space="preserve">Add policies expiring within renewals.pipeline_days to the pipeline; lapse renewals past the grace period</t>
@@ -17394,7 +17394,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/policies/:policyId</t>
+    <t xml:space="preserve">/api/renewals/policies/:policyId</t>
   </si>
   <si>
     <t xml:space="preserve">Put one policy into the renewal pipeline (returns the open renewal)</t>
@@ -17430,7 +17430,7 @@
 }</t>
   </si>
   <si>
-    <t xml:space="preserve">/api/policy-renewals/renewals/queue</t>
+    <t xml:space="preserve">/api/renewals/queue</t>
   </si>
   <si>
     <t xml:space="preserve">Renewal pipeline / queue with dashboard counters (search, status, risk, agent, from, to, page, pageSize)</t>
@@ -17916,6 +17916,9 @@
     <t xml:space="preserve">Master &gt; Schedules</t>
   </si>
   <si>
+    <t xml:space="preserve">read:schedules</t>
+  </si>
+  <si>
     <t xml:space="preserve">{
   "success": true,
   "timeZone": "Asia/Manila",
@@ -18287,6 +18290,98 @@
     <t xml:space="preserve">User Management</t>
   </si>
   <si>
+    <t xml:space="preserve">/api/roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List roles with their permissions and user counts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master &gt; User Management &gt; Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "success": true,
+  "data": [
+    {
+      "id": 1,
+      "code": "sales",
+      "name": "Sales &amp; Marketing (Account Executive)",
+      "permissions": [
+        "read:leads"
+      ],
+      "users": 3
+    }
+  ]
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master &gt; User Management &gt; Role &gt; Add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">write:roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "code": "branch-manager",
+  "name": "Branch Manager",
+  "permissions": [
+    "read:leads",
+    "read:policies",
+    "read:reports"
+  ]
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "success": true,
+  "data": {
+    "id": 9,
+    "code": "branch-manager"
+  }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/api/roles/:id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update a role and its permissions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Master &gt; User Management &gt; Role &gt; Edit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "name": "Branch Manager",
+  "permissions": [
+    "read:leads"
+  ]
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete a non-system role with no users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/api/roles/permissions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All permission codes grouped by module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{
+  "success": true,
+  "data": [
+    {
+      "code": "read:leads",
+      "module": "leads",
+      "description": "View leads"
+    }
+  ]
+}</t>
+  </si>
+  <si>
     <t xml:space="preserve">/api/users</t>
   </si>
   <si>
@@ -18506,98 +18601,6 @@
     "userId": "usr_1",
     "status": "active"
   }
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/users/roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">List roles with their permissions and user counts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master &gt; User Management &gt; Role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "success": true,
-  "data": [
-    {
-      "id": 1,
-      "code": "sales",
-      "name": "Sales &amp; Marketing (Account Executive)",
-      "permissions": [
-        "read:leads"
-      ],
-      "users": 3
-    }
-  ]
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a role</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master &gt; User Management &gt; Role &gt; Add</t>
-  </si>
-  <si>
-    <t xml:space="preserve">write:roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "code": "branch-manager",
-  "name": "Branch Manager",
-  "permissions": [
-    "read:leads",
-    "read:policies",
-    "read:reports"
-  ]
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "success": true,
-  "data": {
-    "id": 9,
-    "code": "branch-manager"
-  }
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/users/roles/:id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update a role and its permissions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master &gt; User Management &gt; Role &gt; Edit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "name": "Branch Manager",
-  "permissions": [
-    "read:leads"
-  ]
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delete a non-system role with no users</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/api/users/roles/permissions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All permission codes grouped by module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{
-  "success": true,
-  "data": [
-    {
-      "code": "read:leads",
-      "module": "leads",
-      "description": "View leads"
-    }
-  ]
 }</t>
   </si>
   <si>
@@ -22765,7 +22768,7 @@
         <v>534</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>552</v>
@@ -22780,10 +22783,13 @@
         <v>15</v>
       </c>
       <c r="H128" s="4" t="s">
-        <v>538</v>
+        <v>542</v>
+      </c>
+      <c r="I128" s="4" t="s">
+        <v>555</v>
       </c>
       <c r="J128" s="4" t="s">
-        <v>555</v>
+        <v>544</v>
       </c>
     </row>
     <row r="129">
@@ -22794,7 +22800,7 @@
         <v>534</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>556</v>
@@ -22809,13 +22815,10 @@
         <v>15</v>
       </c>
       <c r="H129" s="4" t="s">
-        <v>542</v>
-      </c>
-      <c r="I129" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="J129" s="4" t="s">
         <v>559</v>
-      </c>
-      <c r="J129" s="4" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="130">
@@ -26511,11 +26514,8 @@
       <c r="H248" s="4" t="s">
         <v>1052</v>
       </c>
-      <c r="I248" s="4" t="s">
+      <c r="J248" s="4" t="s">
         <v>1053</v>
-      </c>
-      <c r="J248" s="4" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="249">
@@ -26526,28 +26526,28 @@
         <v>1048</v>
       </c>
       <c r="C249" s="0" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D249" s="0" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="E249" s="4" t="s">
         <v>1055</v>
       </c>
       <c r="F249" s="4" t="s">
+        <v>1051</v>
+      </c>
+      <c r="G249" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H249" s="4" t="s">
+        <v>1052</v>
+      </c>
+      <c r="I249" s="4" t="s">
         <v>1056</v>
       </c>
-      <c r="G249" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H249" s="4" t="s">
-        <v>1057</v>
-      </c>
-      <c r="I249" s="4" t="s">
-        <v>1058</v>
-      </c>
       <c r="J249" s="4" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="250">
@@ -26561,13 +26561,13 @@
         <v>11</v>
       </c>
       <c r="D250" s="0" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="E250" s="4" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="F250" s="4" t="s">
-        <v>1062</v>
+        <v>1051</v>
       </c>
       <c r="G250" s="0" t="s">
         <v>15</v>
@@ -26575,8 +26575,11 @@
       <c r="H250" s="4" t="s">
         <v>1052</v>
       </c>
+      <c r="I250" s="4" t="s">
+        <v>1059</v>
+      </c>
       <c r="J250" s="4" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="251">
@@ -26587,28 +26590,28 @@
         <v>1048</v>
       </c>
       <c r="C251" s="0" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D251" s="0" t="s">
-        <v>1060</v>
+        <v>1057</v>
       </c>
       <c r="E251" s="4" t="s">
+        <v>1061</v>
+      </c>
+      <c r="F251" s="4" t="s">
+        <v>1062</v>
+      </c>
+      <c r="G251" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H251" s="4" t="s">
         <v>1063</v>
       </c>
-      <c r="F251" s="4" t="s">
+      <c r="I251" s="4" t="s">
         <v>1064</v>
       </c>
-      <c r="G251" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H251" s="4" t="s">
-        <v>1057</v>
-      </c>
-      <c r="I251" s="4" t="s">
+      <c r="J251" s="4" t="s">
         <v>1065</v>
-      </c>
-      <c r="J251" s="4" t="s">
-        <v>1059</v>
       </c>
     </row>
     <row r="252">
@@ -26619,25 +26622,25 @@
         <v>1048</v>
       </c>
       <c r="C252" s="0" t="s">
-        <v>269</v>
+        <v>11</v>
       </c>
       <c r="D252" s="0" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="E252" s="4" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="F252" s="4" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="G252" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H252" s="4" t="s">
-        <v>1057</v>
+        <v>1052</v>
       </c>
       <c r="J252" s="4" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="253">
@@ -26648,28 +26651,28 @@
         <v>1048</v>
       </c>
       <c r="C253" s="0" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D253" s="0" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E253" s="4" t="s">
         <v>1069</v>
       </c>
-      <c r="E253" s="4" t="s">
+      <c r="F253" s="4" t="s">
         <v>1070</v>
       </c>
-      <c r="F253" s="4" t="s">
+      <c r="G253" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H253" s="4" t="s">
+        <v>1063</v>
+      </c>
+      <c r="I253" s="4" t="s">
         <v>1071</v>
       </c>
-      <c r="G253" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H253" s="4" t="s">
-        <v>1057</v>
-      </c>
-      <c r="I253" s="4" t="s">
-        <v>1072</v>
-      </c>
       <c r="J253" s="4" t="s">
-        <v>1073</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="254">
@@ -26680,25 +26683,25 @@
         <v>1048</v>
       </c>
       <c r="C254" s="0" t="s">
-        <v>11</v>
+        <v>269</v>
       </c>
       <c r="D254" s="0" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E254" s="4" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F254" s="4" t="s">
+        <v>1073</v>
+      </c>
+      <c r="G254" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H254" s="4" t="s">
+        <v>1063</v>
+      </c>
+      <c r="J254" s="4" t="s">
         <v>1074</v>
-      </c>
-      <c r="E254" s="4" t="s">
-        <v>1075</v>
-      </c>
-      <c r="F254" s="4" t="s">
-        <v>1051</v>
-      </c>
-      <c r="G254" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H254" s="4" t="s">
-        <v>1052</v>
-      </c>
-      <c r="J254" s="4" t="s">
-        <v>1076</v>
       </c>
     </row>
     <row r="255">
@@ -26709,28 +26712,28 @@
         <v>1048</v>
       </c>
       <c r="C255" s="0" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D255" s="0" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E255" s="4" t="s">
+        <v>1076</v>
+      </c>
+      <c r="F255" s="4" t="s">
         <v>1077</v>
       </c>
-      <c r="E255" s="4" t="s">
+      <c r="G255" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H255" s="4" t="s">
+        <v>1063</v>
+      </c>
+      <c r="I255" s="4" t="s">
         <v>1078</v>
       </c>
-      <c r="F255" s="4" t="s">
-        <v>1051</v>
-      </c>
-      <c r="G255" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H255" s="4" t="s">
-        <v>1052</v>
-      </c>
-      <c r="I255" s="4" t="s">
+      <c r="J255" s="4" t="s">
         <v>1079</v>
-      </c>
-      <c r="J255" s="4" t="s">
-        <v>1076</v>
       </c>
     </row>
     <row r="256">
@@ -26794,7 +26797,7 @@
         <v>1087</v>
       </c>
       <c r="J257" s="4" t="s">
-        <v>1076</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="258">
@@ -30372,7 +30375,7 @@
         <v>1474</v>
       </c>
       <c r="I372" s="4" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="J372" s="4" t="s">
         <v>1508</v>
@@ -34388,7 +34391,7 @@
         <v>402</v>
       </c>
       <c r="I502" s="4" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="J502" s="4" t="s">
         <v>1508</v>
@@ -39805,10 +39808,10 @@
         <v>15</v>
       </c>
       <c r="H677" s="4" t="s">
-        <v>148</v>
+        <v>2640</v>
       </c>
       <c r="J677" s="4" t="s">
-        <v>2640</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="678">
@@ -39822,22 +39825,22 @@
         <v>18</v>
       </c>
       <c r="D678" s="0" t="s">
-        <v>2641</v>
+        <v>2642</v>
       </c>
       <c r="E678" s="4" t="s">
-        <v>2642</v>
+        <v>2643</v>
       </c>
       <c r="F678" s="4" t="s">
-        <v>2643</v>
+        <v>2644</v>
       </c>
       <c r="G678" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H678" s="4" t="s">
-        <v>2644</v>
+        <v>2645</v>
       </c>
       <c r="I678" s="4" t="s">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="J678" s="4" t="s">
         <v>188</v>
@@ -39854,22 +39857,22 @@
         <v>31</v>
       </c>
       <c r="D679" s="0" t="s">
-        <v>2646</v>
+        <v>2647</v>
       </c>
       <c r="E679" s="4" t="s">
-        <v>2647</v>
+        <v>2648</v>
       </c>
       <c r="F679" s="4" t="s">
-        <v>2648</v>
+        <v>2649</v>
       </c>
       <c r="G679" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H679" s="4" t="s">
-        <v>2644</v>
+        <v>2645</v>
       </c>
       <c r="J679" s="4" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="680">
@@ -39883,22 +39886,22 @@
         <v>11</v>
       </c>
       <c r="D680" s="0" t="s">
-        <v>2650</v>
+        <v>2651</v>
       </c>
       <c r="E680" s="4" t="s">
-        <v>2651</v>
+        <v>2652</v>
       </c>
       <c r="F680" s="4" t="s">
-        <v>2652</v>
+        <v>2653</v>
       </c>
       <c r="G680" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H680" s="4" t="s">
-        <v>148</v>
+        <v>2640</v>
       </c>
       <c r="J680" s="4" t="s">
-        <v>2653</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="681">
@@ -39906,19 +39909,19 @@
         <v>680</v>
       </c>
       <c r="B681" s="0" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="C681" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D681" s="0" t="s">
-        <v>2655</v>
+        <v>2656</v>
       </c>
       <c r="E681" s="4" t="s">
-        <v>2656</v>
+        <v>2657</v>
       </c>
       <c r="F681" s="4" t="s">
-        <v>2657</v>
+        <v>2658</v>
       </c>
       <c r="G681" s="0" t="s">
         <v>15</v>
@@ -39927,10 +39930,10 @@
         <v>148</v>
       </c>
       <c r="I681" s="4" t="s">
-        <v>2658</v>
+        <v>2659</v>
       </c>
       <c r="J681" s="4" t="s">
-        <v>2659</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="682">
@@ -39938,19 +39941,19 @@
         <v>681</v>
       </c>
       <c r="B682" s="0" t="s">
-        <v>2660</v>
+        <v>2661</v>
       </c>
       <c r="C682" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D682" s="0" t="s">
-        <v>2661</v>
+        <v>2662</v>
       </c>
       <c r="E682" s="4" t="s">
-        <v>2662</v>
+        <v>2663</v>
       </c>
       <c r="F682" s="4" t="s">
-        <v>2663</v>
+        <v>2664</v>
       </c>
       <c r="G682" s="0" t="s">
         <v>186</v>
@@ -39959,7 +39962,7 @@
         <v>186</v>
       </c>
       <c r="J682" s="4" t="s">
-        <v>2664</v>
+        <v>2665</v>
       </c>
     </row>
     <row r="683">
@@ -39967,19 +39970,19 @@
         <v>682</v>
       </c>
       <c r="B683" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C683" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D683" s="0" t="s">
-        <v>2666</v>
+        <v>2667</v>
       </c>
       <c r="E683" s="4" t="s">
-        <v>2667</v>
+        <v>2668</v>
       </c>
       <c r="F683" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="G683" s="0" t="s">
         <v>15</v>
@@ -39988,10 +39991,10 @@
         <v>148</v>
       </c>
       <c r="I683" s="4" t="s">
-        <v>2669</v>
+        <v>2670</v>
       </c>
       <c r="J683" s="4" t="s">
-        <v>2670</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="684">
@@ -39999,28 +40002,28 @@
         <v>683</v>
       </c>
       <c r="B684" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C684" s="0" t="s">
         <v>18</v>
       </c>
       <c r="D684" s="0" t="s">
-        <v>2666</v>
+        <v>2667</v>
       </c>
       <c r="E684" s="4" t="s">
-        <v>2671</v>
+        <v>2672</v>
       </c>
       <c r="F684" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="G684" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H684" s="4" t="s">
-        <v>2672</v>
+        <v>2673</v>
       </c>
       <c r="I684" s="4" t="s">
-        <v>2673</v>
+        <v>2674</v>
       </c>
       <c r="J684" s="4" t="s">
         <v>188</v>
@@ -40031,31 +40034,31 @@
         <v>684</v>
       </c>
       <c r="B685" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C685" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D685" s="0" t="s">
-        <v>2674</v>
+        <v>2675</v>
       </c>
       <c r="E685" s="4" t="s">
-        <v>2675</v>
+        <v>2676</v>
       </c>
       <c r="F685" s="4" t="s">
-        <v>2676</v>
+        <v>2677</v>
       </c>
       <c r="G685" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H685" s="4" t="s">
-        <v>2677</v>
+        <v>2678</v>
       </c>
       <c r="I685" s="4" t="s">
-        <v>2678</v>
+        <v>2679</v>
       </c>
       <c r="J685" s="4" t="s">
-        <v>2679</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="686">
@@ -40063,16 +40066,16 @@
         <v>685</v>
       </c>
       <c r="B686" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C686" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D686" s="0" t="s">
-        <v>2680</v>
+        <v>2681</v>
       </c>
       <c r="E686" s="4" t="s">
-        <v>2681</v>
+        <v>2682</v>
       </c>
       <c r="F686" s="4" t="s">
         <v>191</v>
@@ -40084,7 +40087,7 @@
         <v>186</v>
       </c>
       <c r="J686" s="4" t="s">
-        <v>2682</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="687">
@@ -40092,19 +40095,19 @@
         <v>686</v>
       </c>
       <c r="B687" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C687" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D687" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E687" s="4" t="s">
-        <v>2684</v>
+        <v>2685</v>
       </c>
       <c r="F687" s="4" t="s">
-        <v>2685</v>
+        <v>2686</v>
       </c>
       <c r="G687" s="0" t="s">
         <v>186</v>
@@ -40113,7 +40116,7 @@
         <v>186</v>
       </c>
       <c r="J687" s="4" t="s">
-        <v>2686</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="688">
@@ -40121,19 +40124,19 @@
         <v>687</v>
       </c>
       <c r="B688" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C688" s="0" t="s">
         <v>18</v>
       </c>
       <c r="D688" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E688" s="4" t="s">
-        <v>2687</v>
+        <v>2688</v>
       </c>
       <c r="F688" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="G688" s="0" t="s">
         <v>15</v>
@@ -40142,10 +40145,10 @@
         <v>796</v>
       </c>
       <c r="I688" s="4" t="s">
-        <v>2688</v>
+        <v>2689</v>
       </c>
       <c r="J688" s="4" t="s">
-        <v>2686</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="689">
@@ -40153,16 +40156,16 @@
         <v>688</v>
       </c>
       <c r="B689" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C689" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D689" s="0" t="s">
-        <v>2689</v>
+        <v>2690</v>
       </c>
       <c r="E689" s="4" t="s">
-        <v>2690</v>
+        <v>2691</v>
       </c>
       <c r="F689" s="4" t="s">
         <v>1101</v>
@@ -40174,10 +40177,10 @@
         <v>788</v>
       </c>
       <c r="I689" s="4" t="s">
-        <v>2669</v>
+        <v>2670</v>
       </c>
       <c r="J689" s="4" t="s">
-        <v>2691</v>
+        <v>2692</v>
       </c>
     </row>
     <row r="690">
@@ -40185,16 +40188,16 @@
         <v>689</v>
       </c>
       <c r="B690" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C690" s="0" t="s">
         <v>18</v>
       </c>
       <c r="D690" s="0" t="s">
-        <v>2689</v>
+        <v>2690</v>
       </c>
       <c r="E690" s="4" t="s">
-        <v>2692</v>
+        <v>2693</v>
       </c>
       <c r="F690" s="4" t="s">
         <v>1101</v>
@@ -40206,10 +40209,10 @@
         <v>796</v>
       </c>
       <c r="I690" s="4" t="s">
-        <v>2693</v>
+        <v>2694</v>
       </c>
       <c r="J690" s="4" t="s">
-        <v>2694</v>
+        <v>2695</v>
       </c>
     </row>
     <row r="691">
@@ -40217,19 +40220,19 @@
         <v>690</v>
       </c>
       <c r="B691" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C691" s="0" t="s">
         <v>31</v>
       </c>
       <c r="D691" s="0" t="s">
-        <v>2695</v>
+        <v>2696</v>
       </c>
       <c r="E691" s="4" t="s">
-        <v>2696</v>
+        <v>2697</v>
       </c>
       <c r="F691" s="4" t="s">
-        <v>2697</v>
+        <v>2698</v>
       </c>
       <c r="G691" s="0" t="s">
         <v>15</v>
@@ -40238,10 +40241,10 @@
         <v>796</v>
       </c>
       <c r="I691" s="4" t="s">
-        <v>2698</v>
+        <v>2699</v>
       </c>
       <c r="J691" s="4" t="s">
-        <v>2686</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="692">
@@ -40249,19 +40252,19 @@
         <v>691</v>
       </c>
       <c r="B692" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C692" s="0" t="s">
         <v>269</v>
       </c>
       <c r="D692" s="0" t="s">
-        <v>2699</v>
+        <v>2700</v>
       </c>
       <c r="E692" s="4" t="s">
-        <v>2700</v>
+        <v>2701</v>
       </c>
       <c r="F692" s="4" t="s">
-        <v>2701</v>
+        <v>2702</v>
       </c>
       <c r="G692" s="0" t="s">
         <v>15</v>
@@ -40270,7 +40273,7 @@
         <v>796</v>
       </c>
       <c r="J692" s="4" t="s">
-        <v>2686</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="693">
@@ -40278,19 +40281,19 @@
         <v>692</v>
       </c>
       <c r="B693" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="C693" s="0" t="s">
         <v>31</v>
       </c>
       <c r="D693" s="0" t="s">
-        <v>2702</v>
+        <v>2703</v>
       </c>
       <c r="E693" s="4" t="s">
-        <v>2703</v>
+        <v>2704</v>
       </c>
       <c r="F693" s="4" t="s">
-        <v>2704</v>
+        <v>2705</v>
       </c>
       <c r="G693" s="0" t="s">
         <v>15</v>
@@ -40299,10 +40302,10 @@
         <v>796</v>
       </c>
       <c r="I693" s="4" t="s">
-        <v>2705</v>
+        <v>2706</v>
       </c>
       <c r="J693" s="4" t="s">
-        <v>2686</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="694">
@@ -40310,31 +40313,28 @@
         <v>693</v>
       </c>
       <c r="B694" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C694" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D694" s="0" t="s">
-        <v>2707</v>
+        <v>2708</v>
       </c>
       <c r="E694" s="4" t="s">
-        <v>2708</v>
+        <v>2709</v>
       </c>
       <c r="F694" s="4" t="s">
-        <v>2709</v>
+        <v>2710</v>
       </c>
       <c r="G694" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H694" s="4" t="s">
-        <v>2710</v>
-      </c>
-      <c r="I694" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="J694" s="4" t="s">
         <v>2711</v>
-      </c>
-      <c r="J694" s="4" t="s">
-        <v>2712</v>
       </c>
     </row>
     <row r="695">
@@ -40342,31 +40342,31 @@
         <v>694</v>
       </c>
       <c r="B695" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C695" s="0" t="s">
         <v>31</v>
       </c>
       <c r="D695" s="0" t="s">
-        <v>2707</v>
+        <v>2708</v>
       </c>
       <c r="E695" s="4" t="s">
+        <v>2712</v>
+      </c>
+      <c r="F695" s="4" t="s">
         <v>2713</v>
       </c>
-      <c r="F695" s="4" t="s">
+      <c r="G695" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H695" s="4" t="s">
         <v>2714</v>
       </c>
-      <c r="G695" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H695" s="4" t="s">
+      <c r="I695" s="4" t="s">
         <v>2715</v>
       </c>
-      <c r="I695" s="4" t="s">
+      <c r="J695" s="4" t="s">
         <v>2716</v>
-      </c>
-      <c r="J695" s="4" t="s">
-        <v>2717</v>
       </c>
     </row>
     <row r="696">
@@ -40374,28 +40374,31 @@
         <v>695</v>
       </c>
       <c r="B696" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C696" s="0" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D696" s="0" t="s">
+        <v>2717</v>
+      </c>
+      <c r="E696" s="4" t="s">
         <v>2718</v>
       </c>
-      <c r="E696" s="4" t="s">
+      <c r="F696" s="4" t="s">
         <v>2719</v>
       </c>
-      <c r="F696" s="4" t="s">
+      <c r="G696" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H696" s="4" t="s">
+        <v>2714</v>
+      </c>
+      <c r="I696" s="4" t="s">
         <v>2720</v>
       </c>
-      <c r="G696" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H696" s="4" t="s">
-        <v>2710</v>
-      </c>
       <c r="J696" s="4" t="s">
-        <v>2721</v>
+        <v>188</v>
       </c>
     </row>
     <row r="697">
@@ -40403,28 +40406,25 @@
         <v>696</v>
       </c>
       <c r="B697" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C697" s="0" t="s">
-        <v>18</v>
+        <v>269</v>
       </c>
       <c r="D697" s="0" t="s">
-        <v>2718</v>
+        <v>2717</v>
       </c>
       <c r="E697" s="4" t="s">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="F697" s="4" t="s">
-        <v>2723</v>
+        <v>2710</v>
       </c>
       <c r="G697" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H697" s="4" t="s">
-        <v>2715</v>
-      </c>
-      <c r="I697" s="4" t="s">
-        <v>2724</v>
+        <v>2714</v>
       </c>
       <c r="J697" s="4" t="s">
         <v>188</v>
@@ -40435,28 +40435,28 @@
         <v>697</v>
       </c>
       <c r="B698" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C698" s="0" t="s">
-        <v>269</v>
+        <v>11</v>
       </c>
       <c r="D698" s="0" t="s">
-        <v>2718</v>
+        <v>2722</v>
       </c>
       <c r="E698" s="4" t="s">
-        <v>2725</v>
+        <v>2723</v>
       </c>
       <c r="F698" s="4" t="s">
-        <v>2709</v>
+        <v>2713</v>
       </c>
       <c r="G698" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H698" s="4" t="s">
-        <v>2715</v>
+        <v>148</v>
       </c>
       <c r="J698" s="4" t="s">
-        <v>188</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="699">
@@ -40464,28 +40464,31 @@
         <v>698</v>
       </c>
       <c r="B699" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C699" s="0" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D699" s="0" t="s">
+        <v>2725</v>
+      </c>
+      <c r="E699" s="4" t="s">
         <v>2726</v>
       </c>
-      <c r="E699" s="4" t="s">
+      <c r="F699" s="4" t="s">
         <v>2727</v>
       </c>
-      <c r="F699" s="4" t="s">
-        <v>2723</v>
-      </c>
       <c r="G699" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H699" s="4" t="s">
-        <v>2715</v>
+        <v>2728</v>
+      </c>
+      <c r="I699" s="4" t="s">
+        <v>2729</v>
       </c>
       <c r="J699" s="4" t="s">
-        <v>2728</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="700">
@@ -40493,31 +40496,31 @@
         <v>699</v>
       </c>
       <c r="B700" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C700" s="0" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D700" s="0" t="s">
-        <v>2729</v>
+        <v>2725</v>
       </c>
       <c r="E700" s="4" t="s">
-        <v>2730</v>
+        <v>2731</v>
       </c>
       <c r="F700" s="4" t="s">
-        <v>2731</v>
+        <v>2732</v>
       </c>
       <c r="G700" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H700" s="4" t="s">
-        <v>2710</v>
+        <v>2733</v>
       </c>
       <c r="I700" s="4" t="s">
-        <v>2732</v>
+        <v>2734</v>
       </c>
       <c r="J700" s="4" t="s">
-        <v>2733</v>
+        <v>2735</v>
       </c>
     </row>
     <row r="701">
@@ -40525,31 +40528,28 @@
         <v>700</v>
       </c>
       <c r="B701" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C701" s="0" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D701" s="0" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="E701" s="4" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
       <c r="F701" s="4" t="s">
-        <v>2723</v>
+        <v>2738</v>
       </c>
       <c r="G701" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H701" s="4" t="s">
-        <v>2715</v>
-      </c>
-      <c r="I701" s="4" t="s">
-        <v>2736</v>
+        <v>2728</v>
       </c>
       <c r="J701" s="4" t="s">
-        <v>2737</v>
+        <v>2739</v>
       </c>
     </row>
     <row r="702">
@@ -40557,31 +40557,31 @@
         <v>701</v>
       </c>
       <c r="B702" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C702" s="0" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D702" s="0" t="s">
-        <v>2738</v>
+        <v>2736</v>
       </c>
       <c r="E702" s="4" t="s">
-        <v>2739</v>
+        <v>2740</v>
       </c>
       <c r="F702" s="4" t="s">
-        <v>2740</v>
+        <v>2741</v>
       </c>
       <c r="G702" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H702" s="4" t="s">
-        <v>2715</v>
+        <v>2733</v>
       </c>
       <c r="I702" s="4" t="s">
-        <v>2741</v>
+        <v>2742</v>
       </c>
       <c r="J702" s="4" t="s">
-        <v>2742</v>
+        <v>188</v>
       </c>
     </row>
     <row r="703">
@@ -40589,31 +40589,28 @@
         <v>702</v>
       </c>
       <c r="B703" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C703" s="0" t="s">
-        <v>571</v>
+        <v>269</v>
       </c>
       <c r="D703" s="0" t="s">
+        <v>2736</v>
+      </c>
+      <c r="E703" s="4" t="s">
         <v>2743</v>
       </c>
-      <c r="E703" s="4" t="s">
-        <v>2744</v>
-      </c>
       <c r="F703" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="G703" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H703" s="4" t="s">
-        <v>2715</v>
-      </c>
-      <c r="I703" s="4" t="s">
-        <v>2745</v>
+        <v>2733</v>
       </c>
       <c r="J703" s="4" t="s">
-        <v>2746</v>
+        <v>188</v>
       </c>
     </row>
     <row r="704">
@@ -40621,28 +40618,28 @@
         <v>703</v>
       </c>
       <c r="B704" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C704" s="0" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D704" s="0" t="s">
-        <v>2747</v>
+        <v>2744</v>
       </c>
       <c r="E704" s="4" t="s">
-        <v>2748</v>
+        <v>2745</v>
       </c>
       <c r="F704" s="4" t="s">
-        <v>2749</v>
+        <v>2741</v>
       </c>
       <c r="G704" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H704" s="4" t="s">
-        <v>148</v>
+        <v>2733</v>
       </c>
       <c r="J704" s="4" t="s">
-        <v>2750</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="705">
@@ -40650,31 +40647,31 @@
         <v>704</v>
       </c>
       <c r="B705" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C705" s="0" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D705" s="0" t="s">
         <v>2747</v>
       </c>
       <c r="E705" s="4" t="s">
+        <v>2748</v>
+      </c>
+      <c r="F705" s="4" t="s">
+        <v>2749</v>
+      </c>
+      <c r="G705" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H705" s="4" t="s">
+        <v>2728</v>
+      </c>
+      <c r="I705" s="4" t="s">
+        <v>2750</v>
+      </c>
+      <c r="J705" s="4" t="s">
         <v>2751</v>
-      </c>
-      <c r="F705" s="4" t="s">
-        <v>2752</v>
-      </c>
-      <c r="G705" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H705" s="4" t="s">
-        <v>2753</v>
-      </c>
-      <c r="I705" s="4" t="s">
-        <v>2754</v>
-      </c>
-      <c r="J705" s="4" t="s">
-        <v>2755</v>
       </c>
     </row>
     <row r="706">
@@ -40682,31 +40679,31 @@
         <v>705</v>
       </c>
       <c r="B706" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C706" s="0" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D706" s="0" t="s">
-        <v>2756</v>
+        <v>2752</v>
       </c>
       <c r="E706" s="4" t="s">
-        <v>2757</v>
+        <v>2753</v>
       </c>
       <c r="F706" s="4" t="s">
-        <v>2758</v>
+        <v>2741</v>
       </c>
       <c r="G706" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H706" s="4" t="s">
-        <v>2753</v>
+        <v>2733</v>
       </c>
       <c r="I706" s="4" t="s">
-        <v>2759</v>
+        <v>2754</v>
       </c>
       <c r="J706" s="4" t="s">
-        <v>188</v>
+        <v>2755</v>
       </c>
     </row>
     <row r="707">
@@ -40714,28 +40711,31 @@
         <v>706</v>
       </c>
       <c r="B707" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C707" s="0" t="s">
-        <v>269</v>
+        <v>31</v>
       </c>
       <c r="D707" s="0" t="s">
         <v>2756</v>
       </c>
       <c r="E707" s="4" t="s">
+        <v>2757</v>
+      </c>
+      <c r="F707" s="4" t="s">
+        <v>2758</v>
+      </c>
+      <c r="G707" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="H707" s="4" t="s">
+        <v>2733</v>
+      </c>
+      <c r="I707" s="4" t="s">
+        <v>2759</v>
+      </c>
+      <c r="J707" s="4" t="s">
         <v>2760</v>
-      </c>
-      <c r="F707" s="4" t="s">
-        <v>2749</v>
-      </c>
-      <c r="G707" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H707" s="4" t="s">
-        <v>2753</v>
-      </c>
-      <c r="J707" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="708">
@@ -40743,10 +40743,10 @@
         <v>707</v>
       </c>
       <c r="B708" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C708" s="0" t="s">
-        <v>11</v>
+        <v>571</v>
       </c>
       <c r="D708" s="0" t="s">
         <v>2761</v>
@@ -40755,16 +40755,19 @@
         <v>2762</v>
       </c>
       <c r="F708" s="4" t="s">
-        <v>2752</v>
+        <v>2727</v>
       </c>
       <c r="G708" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H708" s="4" t="s">
-        <v>148</v>
+        <v>2733</v>
+      </c>
+      <c r="I708" s="4" t="s">
+        <v>2763</v>
       </c>
       <c r="J708" s="4" t="s">
-        <v>2763</v>
+        <v>2764</v>
       </c>
     </row>
     <row r="709">
@@ -40772,28 +40775,28 @@
         <v>708</v>
       </c>
       <c r="B709" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="C709" s="0" t="s">
         <v>11</v>
       </c>
       <c r="D709" s="0" t="s">
-        <v>2764</v>
+        <v>2765</v>
       </c>
       <c r="E709" s="4" t="s">
-        <v>2765</v>
+        <v>2766</v>
       </c>
       <c r="F709" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="G709" s="0" t="s">
         <v>15</v>
       </c>
       <c r="H709" s="4" t="s">
-        <v>2710</v>
+        <v>2728</v>
       </c>
       <c r="J709" s="4" t="s">
-        <v>2766</v>
+        <v>2767</v>
       </c>
     </row>
   </sheetData>
@@ -40821,7 +40824,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2767</v>
+        <v>2768</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -40836,7 +40839,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>2768</v>
+        <v>2769</v>
       </c>
     </row>
     <row r="2">
@@ -42244,7 +42247,7 @@
     </row>
     <row r="63">
       <c r="A63" s="4" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B63" s="5">
         <v>1</v>
@@ -42253,16 +42256,16 @@
         <v>11</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E63" s="0" t="s">
         <v>534</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="G63" s="5">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="64">
@@ -44383,7 +44386,7 @@
     </row>
     <row r="156">
       <c r="A156" s="4" t="s">
-        <v>2769</v>
+        <v>2770</v>
       </c>
       <c r="B156" s="5">
         <v>1</v>
@@ -45142,7 +45145,7 @@
     </row>
     <row r="189">
       <c r="A189" s="4" t="s">
-        <v>2770</v>
+        <v>2771</v>
       </c>
       <c r="B189" s="5">
         <v>1</v>
@@ -46568,7 +46571,7 @@
     </row>
     <row r="251">
       <c r="A251" s="4" t="s">
-        <v>2771</v>
+        <v>2772</v>
       </c>
       <c r="B251" s="5">
         <v>1</v>
@@ -46867,7 +46870,7 @@
     </row>
     <row r="264">
       <c r="A264" s="4" t="s">
-        <v>2772</v>
+        <v>2773</v>
       </c>
       <c r="B264" s="5">
         <v>1</v>
@@ -47074,7 +47077,7 @@
     </row>
     <row r="273">
       <c r="A273" s="4" t="s">
-        <v>2773</v>
+        <v>2774</v>
       </c>
       <c r="B273" s="5">
         <v>1</v>
@@ -47083,13 +47086,13 @@
         <v>11</v>
       </c>
       <c r="D273" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E273" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F273" s="4" t="s">
-        <v>2684</v>
+        <v>2685</v>
       </c>
       <c r="G273" s="5">
         <v>686</v>
@@ -47120,7 +47123,7 @@
     </row>
     <row r="275">
       <c r="A275" s="4" t="s">
-        <v>2774</v>
+        <v>2775</v>
       </c>
       <c r="B275" s="5">
         <v>1</v>
@@ -47143,7 +47146,7 @@
     </row>
     <row r="276">
       <c r="A276" s="4" t="s">
-        <v>2775</v>
+        <v>2776</v>
       </c>
       <c r="B276" s="5">
         <v>1</v>
@@ -47557,7 +47560,7 @@
     </row>
     <row r="294">
       <c r="A294" s="4" t="s">
-        <v>2776</v>
+        <v>2777</v>
       </c>
       <c r="B294" s="5">
         <v>2</v>
@@ -47580,7 +47583,7 @@
     </row>
     <row r="295">
       <c r="A295" s="4" t="s">
-        <v>2776</v>
+        <v>2777</v>
       </c>
       <c r="B295" s="5">
         <v>2</v>
@@ -47902,7 +47905,7 @@
     </row>
     <row r="309">
       <c r="A309" s="4" t="s">
-        <v>2777</v>
+        <v>2778</v>
       </c>
       <c r="B309" s="5">
         <v>1</v>
@@ -47925,7 +47928,7 @@
     </row>
     <row r="310">
       <c r="A310" s="4" t="s">
-        <v>2778</v>
+        <v>2779</v>
       </c>
       <c r="B310" s="5">
         <v>1</v>
@@ -48017,7 +48020,7 @@
     </row>
     <row r="314">
       <c r="A314" s="4" t="s">
-        <v>2657</v>
+        <v>2658</v>
       </c>
       <c r="B314" s="5">
         <v>1</v>
@@ -48026,13 +48029,13 @@
         <v>11</v>
       </c>
       <c r="D314" s="0" t="s">
+        <v>2656</v>
+      </c>
+      <c r="E314" s="0" t="s">
         <v>2655</v>
       </c>
-      <c r="E314" s="0" t="s">
-        <v>2654</v>
-      </c>
       <c r="F314" s="4" t="s">
-        <v>2656</v>
+        <v>2657</v>
       </c>
       <c r="G314" s="5">
         <v>680</v>
@@ -48040,7 +48043,7 @@
     </row>
     <row r="315">
       <c r="A315" s="4" t="s">
-        <v>2779</v>
+        <v>2780</v>
       </c>
       <c r="B315" s="5">
         <v>1</v>
@@ -48063,7 +48066,7 @@
     </row>
     <row r="316">
       <c r="A316" s="4" t="s">
-        <v>2780</v>
+        <v>2781</v>
       </c>
       <c r="B316" s="5">
         <v>1</v>
@@ -48293,7 +48296,7 @@
     </row>
     <row r="326">
       <c r="A326" s="4" t="s">
-        <v>2676</v>
+        <v>2677</v>
       </c>
       <c r="B326" s="5">
         <v>1</v>
@@ -48302,13 +48305,13 @@
         <v>11</v>
       </c>
       <c r="D326" s="0" t="s">
-        <v>2674</v>
+        <v>2675</v>
       </c>
       <c r="E326" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F326" s="4" t="s">
-        <v>2675</v>
+        <v>2676</v>
       </c>
       <c r="G326" s="5">
         <v>684</v>
@@ -48371,13 +48374,13 @@
         <v>11</v>
       </c>
       <c r="D329" s="0" t="s">
-        <v>2689</v>
+        <v>2690</v>
       </c>
       <c r="E329" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F329" s="4" t="s">
-        <v>2690</v>
+        <v>2691</v>
       </c>
       <c r="G329" s="5">
         <v>688</v>
@@ -48394,13 +48397,13 @@
         <v>18</v>
       </c>
       <c r="D330" s="0" t="s">
-        <v>2689</v>
+        <v>2690</v>
       </c>
       <c r="E330" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F330" s="4" t="s">
-        <v>2692</v>
+        <v>2693</v>
       </c>
       <c r="G330" s="5">
         <v>689</v>
@@ -48937,7 +48940,7 @@
     </row>
     <row r="354">
       <c r="A354" s="4" t="s">
-        <v>2781</v>
+        <v>2782</v>
       </c>
       <c r="B354" s="5">
         <v>1</v>
@@ -49857,7 +49860,7 @@
     </row>
     <row r="394">
       <c r="A394" s="4" t="s">
-        <v>2643</v>
+        <v>2644</v>
       </c>
       <c r="B394" s="5">
         <v>1</v>
@@ -49866,13 +49869,13 @@
         <v>18</v>
       </c>
       <c r="D394" s="0" t="s">
-        <v>2641</v>
+        <v>2642</v>
       </c>
       <c r="E394" s="0" t="s">
         <v>2636</v>
       </c>
       <c r="F394" s="4" t="s">
-        <v>2642</v>
+        <v>2643</v>
       </c>
       <c r="G394" s="5">
         <v>677</v>
@@ -49880,7 +49883,7 @@
     </row>
     <row r="395">
       <c r="A395" s="4" t="s">
-        <v>2652</v>
+        <v>2653</v>
       </c>
       <c r="B395" s="5">
         <v>1</v>
@@ -49889,13 +49892,13 @@
         <v>11</v>
       </c>
       <c r="D395" s="0" t="s">
-        <v>2650</v>
+        <v>2651</v>
       </c>
       <c r="E395" s="0" t="s">
         <v>2636</v>
       </c>
       <c r="F395" s="4" t="s">
-        <v>2651</v>
+        <v>2652</v>
       </c>
       <c r="G395" s="5">
         <v>679</v>
@@ -49903,7 +49906,7 @@
     </row>
     <row r="396">
       <c r="A396" s="4" t="s">
-        <v>2648</v>
+        <v>2649</v>
       </c>
       <c r="B396" s="5">
         <v>1</v>
@@ -49912,13 +49915,13 @@
         <v>31</v>
       </c>
       <c r="D396" s="0" t="s">
-        <v>2646</v>
+        <v>2647</v>
       </c>
       <c r="E396" s="0" t="s">
         <v>2636</v>
       </c>
       <c r="F396" s="4" t="s">
-        <v>2647</v>
+        <v>2648</v>
       </c>
       <c r="G396" s="5">
         <v>678</v>
@@ -49926,7 +49929,7 @@
     </row>
     <row r="397">
       <c r="A397" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="B397" s="5">
         <v>4</v>
@@ -49935,13 +49938,13 @@
         <v>11</v>
       </c>
       <c r="D397" s="0" t="s">
+        <v>2667</v>
+      </c>
+      <c r="E397" s="0" t="s">
         <v>2666</v>
       </c>
-      <c r="E397" s="0" t="s">
-        <v>2665</v>
-      </c>
       <c r="F397" s="4" t="s">
-        <v>2667</v>
+        <v>2668</v>
       </c>
       <c r="G397" s="5">
         <v>682</v>
@@ -49949,7 +49952,7 @@
     </row>
     <row r="398">
       <c r="A398" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="B398" s="5">
         <v>4</v>
@@ -49958,13 +49961,13 @@
         <v>18</v>
       </c>
       <c r="D398" s="0" t="s">
+        <v>2667</v>
+      </c>
+      <c r="E398" s="0" t="s">
         <v>2666</v>
       </c>
-      <c r="E398" s="0" t="s">
-        <v>2665</v>
-      </c>
       <c r="F398" s="4" t="s">
-        <v>2671</v>
+        <v>2672</v>
       </c>
       <c r="G398" s="5">
         <v>683</v>
@@ -49972,7 +49975,7 @@
     </row>
     <row r="399">
       <c r="A399" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="B399" s="5">
         <v>4</v>
@@ -49981,13 +49984,13 @@
         <v>11</v>
       </c>
       <c r="D399" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E399" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F399" s="4" t="s">
-        <v>2684</v>
+        <v>2685</v>
       </c>
       <c r="G399" s="5">
         <v>686</v>
@@ -49995,7 +49998,7 @@
     </row>
     <row r="400">
       <c r="A400" s="4" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="B400" s="5">
         <v>4</v>
@@ -50004,13 +50007,13 @@
         <v>18</v>
       </c>
       <c r="D400" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E400" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F400" s="4" t="s">
-        <v>2687</v>
+        <v>2688</v>
       </c>
       <c r="G400" s="5">
         <v>687</v>
@@ -50018,7 +50021,7 @@
     </row>
     <row r="401">
       <c r="A401" s="4" t="s">
-        <v>2697</v>
+        <v>2698</v>
       </c>
       <c r="B401" s="5">
         <v>1</v>
@@ -50027,13 +50030,13 @@
         <v>31</v>
       </c>
       <c r="D401" s="0" t="s">
-        <v>2695</v>
+        <v>2696</v>
       </c>
       <c r="E401" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F401" s="4" t="s">
-        <v>2696</v>
+        <v>2697</v>
       </c>
       <c r="G401" s="5">
         <v>690</v>
@@ -50041,7 +50044,7 @@
     </row>
     <row r="402">
       <c r="A402" s="4" t="s">
-        <v>2701</v>
+        <v>2702</v>
       </c>
       <c r="B402" s="5">
         <v>1</v>
@@ -50050,13 +50053,13 @@
         <v>269</v>
       </c>
       <c r="D402" s="0" t="s">
-        <v>2699</v>
+        <v>2700</v>
       </c>
       <c r="E402" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F402" s="4" t="s">
-        <v>2700</v>
+        <v>2701</v>
       </c>
       <c r="G402" s="5">
         <v>691</v>
@@ -50064,7 +50067,7 @@
     </row>
     <row r="403">
       <c r="A403" s="4" t="s">
-        <v>2704</v>
+        <v>2705</v>
       </c>
       <c r="B403" s="5">
         <v>1</v>
@@ -50073,13 +50076,13 @@
         <v>31</v>
       </c>
       <c r="D403" s="0" t="s">
-        <v>2702</v>
+        <v>2703</v>
       </c>
       <c r="E403" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F403" s="4" t="s">
-        <v>2703</v>
+        <v>2704</v>
       </c>
       <c r="G403" s="5">
         <v>692</v>
@@ -50087,7 +50090,7 @@
     </row>
     <row r="404">
       <c r="A404" s="4" t="s">
-        <v>2749</v>
+        <v>2710</v>
       </c>
       <c r="B404" s="5">
         <v>2</v>
@@ -50096,21 +50099,21 @@
         <v>11</v>
       </c>
       <c r="D404" s="0" t="s">
-        <v>2747</v>
+        <v>2708</v>
       </c>
       <c r="E404" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F404" s="4" t="s">
-        <v>2748</v>
+        <v>2709</v>
       </c>
       <c r="G404" s="5">
-        <v>703</v>
+        <v>693</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="4" t="s">
-        <v>2749</v>
+        <v>2710</v>
       </c>
       <c r="B405" s="5">
         <v>2</v>
@@ -50119,21 +50122,21 @@
         <v>269</v>
       </c>
       <c r="D405" s="0" t="s">
-        <v>2756</v>
+        <v>2717</v>
       </c>
       <c r="E405" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F405" s="4" t="s">
-        <v>2760</v>
+        <v>2721</v>
       </c>
       <c r="G405" s="5">
-        <v>706</v>
+        <v>696</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="4" t="s">
-        <v>2752</v>
+        <v>2713</v>
       </c>
       <c r="B406" s="5">
         <v>2</v>
@@ -50142,21 +50145,21 @@
         <v>31</v>
       </c>
       <c r="D406" s="0" t="s">
-        <v>2747</v>
+        <v>2708</v>
       </c>
       <c r="E406" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F406" s="4" t="s">
-        <v>2751</v>
+        <v>2712</v>
       </c>
       <c r="G406" s="5">
-        <v>704</v>
+        <v>694</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="4" t="s">
-        <v>2752</v>
+        <v>2713</v>
       </c>
       <c r="B407" s="5">
         <v>2</v>
@@ -50165,21 +50168,21 @@
         <v>11</v>
       </c>
       <c r="D407" s="0" t="s">
-        <v>2761</v>
+        <v>2722</v>
       </c>
       <c r="E407" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F407" s="4" t="s">
-        <v>2762</v>
+        <v>2723</v>
       </c>
       <c r="G407" s="5">
-        <v>707</v>
+        <v>697</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="4" t="s">
-        <v>2758</v>
+        <v>2719</v>
       </c>
       <c r="B408" s="5">
         <v>1</v>
@@ -50188,21 +50191,21 @@
         <v>18</v>
       </c>
       <c r="D408" s="0" t="s">
-        <v>2756</v>
+        <v>2717</v>
       </c>
       <c r="E408" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F408" s="4" t="s">
-        <v>2757</v>
+        <v>2718</v>
       </c>
       <c r="G408" s="5">
-        <v>705</v>
+        <v>695</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="B409" s="5">
         <v>4</v>
@@ -50211,21 +50214,21 @@
         <v>11</v>
       </c>
       <c r="D409" s="0" t="s">
+        <v>2725</v>
+      </c>
+      <c r="E409" s="0" t="s">
         <v>2707</v>
       </c>
-      <c r="E409" s="0" t="s">
-        <v>2706</v>
-      </c>
       <c r="F409" s="4" t="s">
-        <v>2708</v>
+        <v>2726</v>
       </c>
       <c r="G409" s="5">
-        <v>693</v>
+        <v>698</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="B410" s="5">
         <v>4</v>
@@ -50234,21 +50237,21 @@
         <v>269</v>
       </c>
       <c r="D410" s="0" t="s">
-        <v>2718</v>
+        <v>2736</v>
       </c>
       <c r="E410" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F410" s="4" t="s">
-        <v>2725</v>
+        <v>2743</v>
       </c>
       <c r="G410" s="5">
-        <v>697</v>
+        <v>702</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="B411" s="5">
         <v>4</v>
@@ -50257,21 +50260,21 @@
         <v>571</v>
       </c>
       <c r="D411" s="0" t="s">
-        <v>2743</v>
+        <v>2761</v>
       </c>
       <c r="E411" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F411" s="4" t="s">
-        <v>2744</v>
+        <v>2762</v>
       </c>
       <c r="G411" s="5">
-        <v>702</v>
+        <v>707</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="4" t="s">
-        <v>2709</v>
+        <v>2727</v>
       </c>
       <c r="B412" s="5">
         <v>4</v>
@@ -50280,13 +50283,13 @@
         <v>11</v>
       </c>
       <c r="D412" s="0" t="s">
-        <v>2764</v>
+        <v>2765</v>
       </c>
       <c r="E412" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F412" s="4" t="s">
-        <v>2765</v>
+        <v>2766</v>
       </c>
       <c r="G412" s="5">
         <v>708</v>
@@ -50294,7 +50297,7 @@
     </row>
     <row r="413">
       <c r="A413" s="4" t="s">
-        <v>2714</v>
+        <v>2732</v>
       </c>
       <c r="B413" s="5">
         <v>1</v>
@@ -50303,21 +50306,21 @@
         <v>31</v>
       </c>
       <c r="D413" s="0" t="s">
+        <v>2725</v>
+      </c>
+      <c r="E413" s="0" t="s">
         <v>2707</v>
       </c>
-      <c r="E413" s="0" t="s">
-        <v>2706</v>
-      </c>
       <c r="F413" s="4" t="s">
-        <v>2713</v>
+        <v>2731</v>
       </c>
       <c r="G413" s="5">
-        <v>694</v>
+        <v>699</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="4" t="s">
-        <v>2723</v>
+        <v>2741</v>
       </c>
       <c r="B414" s="5">
         <v>3</v>
@@ -50326,21 +50329,21 @@
         <v>18</v>
       </c>
       <c r="D414" s="0" t="s">
-        <v>2718</v>
+        <v>2736</v>
       </c>
       <c r="E414" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F414" s="4" t="s">
-        <v>2722</v>
+        <v>2740</v>
       </c>
       <c r="G414" s="5">
-        <v>696</v>
+        <v>701</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="4" t="s">
-        <v>2723</v>
+        <v>2741</v>
       </c>
       <c r="B415" s="5">
         <v>3</v>
@@ -50349,21 +50352,21 @@
         <v>31</v>
       </c>
       <c r="D415" s="0" t="s">
-        <v>2726</v>
+        <v>2744</v>
       </c>
       <c r="E415" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F415" s="4" t="s">
-        <v>2727</v>
+        <v>2745</v>
       </c>
       <c r="G415" s="5">
-        <v>698</v>
+        <v>703</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="4" t="s">
-        <v>2723</v>
+        <v>2741</v>
       </c>
       <c r="B416" s="5">
         <v>3</v>
@@ -50372,21 +50375,21 @@
         <v>31</v>
       </c>
       <c r="D416" s="0" t="s">
-        <v>2734</v>
+        <v>2752</v>
       </c>
       <c r="E416" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F416" s="4" t="s">
-        <v>2735</v>
+        <v>2753</v>
       </c>
       <c r="G416" s="5">
-        <v>700</v>
+        <v>705</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="4" t="s">
-        <v>2740</v>
+        <v>2758</v>
       </c>
       <c r="B417" s="5">
         <v>1</v>
@@ -50395,21 +50398,21 @@
         <v>31</v>
       </c>
       <c r="D417" s="0" t="s">
-        <v>2738</v>
+        <v>2756</v>
       </c>
       <c r="E417" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F417" s="4" t="s">
-        <v>2739</v>
+        <v>2757</v>
       </c>
       <c r="G417" s="5">
-        <v>701</v>
+        <v>706</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="4" t="s">
-        <v>2720</v>
+        <v>2738</v>
       </c>
       <c r="B418" s="5">
         <v>1</v>
@@ -50418,21 +50421,21 @@
         <v>11</v>
       </c>
       <c r="D418" s="0" t="s">
-        <v>2718</v>
+        <v>2736</v>
       </c>
       <c r="E418" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F418" s="4" t="s">
-        <v>2719</v>
+        <v>2737</v>
       </c>
       <c r="G418" s="5">
-        <v>695</v>
+        <v>700</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="4" t="s">
-        <v>2731</v>
+        <v>2749</v>
       </c>
       <c r="B419" s="5">
         <v>1</v>
@@ -50441,16 +50444,16 @@
         <v>11</v>
       </c>
       <c r="D419" s="0" t="s">
-        <v>2729</v>
+        <v>2747</v>
       </c>
       <c r="E419" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="F419" s="4" t="s">
-        <v>2730</v>
+        <v>2748</v>
       </c>
       <c r="G419" s="5">
-        <v>699</v>
+        <v>704</v>
       </c>
     </row>
     <row r="420">
@@ -50478,7 +50481,7 @@
     </row>
     <row r="421">
       <c r="A421" s="4" t="s">
-        <v>2663</v>
+        <v>2664</v>
       </c>
       <c r="B421" s="5">
         <v>1</v>
@@ -50487,13 +50490,13 @@
         <v>11</v>
       </c>
       <c r="D421" s="0" t="s">
+        <v>2662</v>
+      </c>
+      <c r="E421" s="0" t="s">
         <v>2661</v>
       </c>
-      <c r="E421" s="0" t="s">
-        <v>2660</v>
-      </c>
       <c r="F421" s="4" t="s">
-        <v>2662</v>
+        <v>2663</v>
       </c>
       <c r="G421" s="5">
         <v>681</v>
@@ -51269,16 +51272,16 @@
         <v>11</v>
       </c>
       <c r="D455" s="0" t="s">
-        <v>1074</v>
+        <v>1054</v>
       </c>
       <c r="E455" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F455" s="4" t="s">
-        <v>1075</v>
+        <v>1055</v>
       </c>
       <c r="G455" s="5">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="456">
@@ -51292,16 +51295,16 @@
         <v>11</v>
       </c>
       <c r="D456" s="0" t="s">
-        <v>1077</v>
+        <v>1057</v>
       </c>
       <c r="E456" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F456" s="4" t="s">
-        <v>1078</v>
+        <v>1058</v>
       </c>
       <c r="G456" s="5">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="457">
@@ -51352,7 +51355,7 @@
     </row>
     <row r="459">
       <c r="A459" s="4" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="B459" s="5">
         <v>1</v>
@@ -51361,21 +51364,21 @@
         <v>31</v>
       </c>
       <c r="D459" s="0" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="E459" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F459" s="4" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="G459" s="5">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="4" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="B460" s="5">
         <v>1</v>
@@ -51384,16 +51387,16 @@
         <v>31</v>
       </c>
       <c r="D460" s="0" t="s">
-        <v>1049</v>
+        <v>1057</v>
       </c>
       <c r="E460" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F460" s="4" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="G460" s="5">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="461">
@@ -51513,7 +51516,7 @@
     </row>
     <row r="466">
       <c r="A466" s="4" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="B466" s="5">
         <v>1</v>
@@ -51522,21 +51525,21 @@
         <v>269</v>
       </c>
       <c r="D466" s="0" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="E466" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F466" s="4" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="G466" s="5">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="4" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="B467" s="5">
         <v>1</v>
@@ -51545,16 +51548,16 @@
         <v>18</v>
       </c>
       <c r="D467" s="0" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="E467" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F467" s="4" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
       <c r="G467" s="5">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="468">
@@ -51582,7 +51585,7 @@
     </row>
     <row r="469">
       <c r="A469" s="4" t="s">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="B469" s="5">
         <v>1</v>
@@ -51591,16 +51594,16 @@
         <v>11</v>
       </c>
       <c r="D469" s="0" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="E469" s="0" t="s">
         <v>1048</v>
       </c>
       <c r="F469" s="4" t="s">
-        <v>1061</v>
+        <v>1067</v>
       </c>
       <c r="G469" s="5">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="470">
@@ -52525,7 +52528,7 @@
     </row>
     <row r="510">
       <c r="A510" s="4" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="B510" s="5">
         <v>1</v>
@@ -52534,16 +52537,16 @@
         <v>31</v>
       </c>
       <c r="D510" s="0" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E510" s="0" t="s">
         <v>534</v>
       </c>
       <c r="F510" s="4" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="G510" s="5">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="511">
@@ -53629,7 +53632,7 @@
     </row>
     <row r="558">
       <c r="A558" s="4" t="s">
-        <v>2782</v>
+        <v>2783</v>
       </c>
       <c r="B558" s="5">
         <v>1</v>
@@ -55009,7 +55012,7 @@
     </row>
     <row r="618">
       <c r="A618" s="4" t="s">
-        <v>2783</v>
+        <v>2784</v>
       </c>
       <c r="B618" s="5">
         <v>1</v>
@@ -55929,7 +55932,7 @@
     </row>
     <row r="658">
       <c r="A658" s="4" t="s">
-        <v>2784</v>
+        <v>2785</v>
       </c>
       <c r="B658" s="5">
         <v>2</v>
@@ -55952,7 +55955,7 @@
     </row>
     <row r="659">
       <c r="A659" s="4" t="s">
-        <v>2784</v>
+        <v>2785</v>
       </c>
       <c r="B659" s="5">
         <v>2</v>
@@ -56136,7 +56139,7 @@
     </row>
     <row r="667">
       <c r="A667" s="4" t="s">
-        <v>2785</v>
+        <v>2786</v>
       </c>
       <c r="B667" s="5">
         <v>1</v>
@@ -56159,7 +56162,7 @@
     </row>
     <row r="668">
       <c r="A668" s="4" t="s">
-        <v>2786</v>
+        <v>2787</v>
       </c>
       <c r="B668" s="5">
         <v>1</v>
@@ -56205,7 +56208,7 @@
     </row>
     <row r="670">
       <c r="A670" s="4" t="s">
-        <v>2787</v>
+        <v>2788</v>
       </c>
       <c r="B670" s="5">
         <v>1</v>
@@ -56780,7 +56783,7 @@
     </row>
     <row r="695">
       <c r="A695" s="4" t="s">
-        <v>2788</v>
+        <v>2789</v>
       </c>
       <c r="B695" s="5">
         <v>2</v>
@@ -56803,7 +56806,7 @@
     </row>
     <row r="696">
       <c r="A696" s="4" t="s">
-        <v>2788</v>
+        <v>2789</v>
       </c>
       <c r="B696" s="5">
         <v>2</v>
@@ -56918,7 +56921,7 @@
     </row>
     <row r="701">
       <c r="A701" s="4" t="s">
-        <v>2789</v>
+        <v>2790</v>
       </c>
       <c r="B701" s="5">
         <v>1</v>
@@ -57286,7 +57289,7 @@
     </row>
     <row r="717">
       <c r="A717" s="4" t="s">
-        <v>2790</v>
+        <v>2791</v>
       </c>
       <c r="B717" s="5">
         <v>1</v>
@@ -57309,7 +57312,7 @@
     </row>
     <row r="718">
       <c r="A718" s="4" t="s">
-        <v>2791</v>
+        <v>2792</v>
       </c>
       <c r="B718" s="5">
         <v>1</v>
@@ -57387,13 +57390,13 @@
         <v>11</v>
       </c>
       <c r="D721" s="0" t="s">
-        <v>2680</v>
+        <v>2681</v>
       </c>
       <c r="E721" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F721" s="4" t="s">
-        <v>2681</v>
+        <v>2682</v>
       </c>
       <c r="G721" s="5">
         <v>685</v>
@@ -57410,13 +57413,13 @@
         <v>11</v>
       </c>
       <c r="D722" s="0" t="s">
-        <v>2683</v>
+        <v>2684</v>
       </c>
       <c r="E722" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="F722" s="4" t="s">
-        <v>2684</v>
+        <v>2685</v>
       </c>
       <c r="G722" s="5">
         <v>686</v>
@@ -57424,7 +57427,7 @@
     </row>
     <row r="723">
       <c r="A723" s="4" t="s">
-        <v>2792</v>
+        <v>2793</v>
       </c>
       <c r="B723" s="5">
         <v>1</v>
@@ -57679,7 +57682,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2793</v>
+        <v>2794</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
@@ -57697,10 +57700,10 @@
         <v>269</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>2794</v>
+        <v>2795</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>2795</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="2">
@@ -58894,7 +58897,7 @@
     </row>
     <row r="43">
       <c r="A43" s="0" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B43" s="5">
         <v>1</v>
@@ -58923,7 +58926,7 @@
     </row>
     <row r="44">
       <c r="A44" s="0" t="s">
-        <v>2660</v>
+        <v>2661</v>
       </c>
       <c r="B44" s="5">
         <v>1</v>
@@ -58952,7 +58955,7 @@
     </row>
     <row r="45">
       <c r="A45" s="0" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="B45" s="5">
         <v>11</v>
@@ -58981,7 +58984,7 @@
     </row>
     <row r="46">
       <c r="A46" s="0" t="s">
-        <v>2706</v>
+        <v>2707</v>
       </c>
       <c r="B46" s="5">
         <v>16</v>
@@ -59010,7 +59013,7 @@
     </row>
     <row r="47">
       <c r="A47" s="0" t="s">
-        <v>2796</v>
+        <v>2797</v>
       </c>
       <c r="B47" s="5">
         <v>708</v>

</xml_diff>

<commit_message>
Regenerate API reference after the screen stability merge
</commit_message>
<xml_diff>
--- a/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
+++ b/backend/docs/api/BrokerVerse_API_Touchpoints.xlsx
@@ -4292,7 +4292,7 @@
     <t xml:space="preserve">/api/clients</t>
   </si>
   <si>
-    <t xml:space="preserve">List clients (search, leadCategory, status; paging)</t>
+    <t xml:space="preserve">List clients (search, leadCategory, clientType individual / corporate, status; paging)</t>
   </si>
   <si>
     <t xml:space="preserve">Operations &gt; Clients</t>
@@ -22736,7 +22736,7 @@
     <t xml:space="preserve">/api/settings/audit</t>
   </si>
   <si>
-    <t xml:space="preserve">Audit trail (filter by entity / entityId / user and a from / to business-date range, general.timezone)</t>
+    <t xml:space="preserve">Audit trail (filter by entity / entityId / user and a from / to business-date range, general.timezone; newest first; with page / pageSize a page of the log and its total, else the latest `limit` entries)</t>
   </si>
   <si>
     <t xml:space="preserve">Master &gt; Audit trail</t>
@@ -22745,7 +22745,7 @@
     <t xml:space="preserve">role:system-admin, read:audit</t>
   </si>
   <si>
-    <t xml:space="preserve">Query: ?entity=policy&amp;entityId=pol_1&amp;username=BrokerVerse&amp;from=2026-09-01&amp;to=2026-09-30&amp;limit=100</t>
+    <t xml:space="preserve">Query: ?entity=policy&amp;entityId=pol_1&amp;username=BrokerVerse&amp;from=2026-09-01&amp;to=2026-09-30&amp;page=1&amp;pageSize=20</t>
   </si>
   <si>
     <t xml:space="preserve">{
@@ -22757,7 +22757,11 @@
       "entity": "policy",
       "action": "create"
     }
-  ]
+  ],
+  "total": 1,
+  "page": 1,
+  "pageSize": 20,
+  "totalPages": 1
 }</t>
   </si>
   <si>

</xml_diff>